<commit_message>
Regenerar resultados ponderados y artefactos
</commit_message>
<xml_diff>
--- a/TABLAS/STROBE_checklist.xlsx
+++ b/TABLAS/STROBE_checklist.xlsx
@@ -614,7 +614,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Materiales y métodos &gt; Diseño y fuente de datos; Resultados &gt; Muestra (n=25 089)</t>
+          <t>Materiales y métodos &gt; Diseño y fuente de datos; Resultados &gt; Muestra (n=25 088)</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Materiales y métodos &gt; Diseño muestral complejo</t>
+          <t>Materiales y métodos &gt; Diseño muestral complejo; Modelo estadístico (pseudo-verosimilitud con ponderador calibrado normalizado dentro de municipio)</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Materiales y métodos &gt; Reclasificación y validación (sensibilidad a matriz de vecindad); Figura S1 (validación cruzada)</t>
+          <t>Materiales y métodos &gt; Reclasificación y validación (sensibilidades a ponderación y matriz de vecindad); Figura S1 (validación cruzada)</t>
         </is>
       </c>
     </row>

</xml_diff>